<commit_message>
Change choiches to "Yes" and "No"
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Dropbox\Uni Oldenburg\#3 - RStudio dateien\#4 - MSAT - main test R script\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD168A17-D284-4D26-9233-AA0CFBA7A43A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83471C14-FC0E-43ED-9944-5FC57D82CA79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1890" windowWidth="38640" windowHeight="20865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t>key</t>
   </si>
@@ -91,18 +91,9 @@
     <t>Bitte gib Deine ID ein</t>
   </si>
   <si>
-    <t>Die ID ist leider ungültig. Bitte versuche es noch mal.</t>
-  </si>
-  <si>
     <t>Weiter</t>
   </si>
   <si>
-    <t>Du hast {{num_correct}} von {{num_question}} Fragen richtig beantwortet.</t>
-  </si>
-  <si>
-    <t>Dein Testergebnis</t>
-  </si>
-  <si>
     <t>Werte</t>
   </si>
   <si>
@@ -133,9 +124,6 @@
     <t>Score</t>
   </si>
   <si>
-    <t>Du hast den Test zur musikalischen Szenenanalyse erfolgreich beendet.</t>
-  </si>
-  <si>
     <t>Musikalische Szenenanalyse Test</t>
   </si>
   <si>
@@ -187,21 +175,12 @@
     <t>MAIN_INTRO</t>
   </si>
   <si>
-    <t>**Übungsfrage 1** \\ Bitte hören Sie sich den folgenden Clip an und entscheiden Sie, ob das Zielinstrument in der Instrumentenmixtur spielte.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
-  </si>
-  <si>
-    <t>**Practice question 1** \\ Please listen to the following clip and and decide, whether the target plays in the mixture.\\ Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
-  </si>
-  <si>
     <t>Nun geht es mit dem Haupttest los, in dem Ihre Antworten gespeichert werden. \\ Ab jetzt bekommen Sie keine Rückmeldung mehr. Viel Erfolg!</t>
   </si>
   <si>
     <t>You are about to start the main test, where your results will be recorded. \\ You won't receive any feedback after individual questions. Good luck and have fun!</t>
   </si>
   <si>
-    <t>Dein Browser unterstützt kein Audio. Dieser Test funktioniert nicht ohne Audio! Probieren Sie es bitte mit einem anderen Browser (bspw. Google Chrome).</t>
-  </si>
-  <si>
     <t>Your browser doesn't support audio. This test won't work without audio, sorry! Pleas try using another Browser (e.g. Google Chrome).</t>
   </si>
   <si>
@@ -209,24 +188,6 @@
   </si>
   <si>
     <t>Welcome to the test for musical scene analysis (MSA)</t>
-  </si>
-  <si>
-    <t>&lt;h4&gt;Willkommen zum Test zur Musikalischen Szenenanalysen (MSA)&lt;/h4&gt; In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. \\ 
-Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Zuerst wirst du Beispiele hören und dann ein paar Übungsaufgaben machen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.\\ If you are not sure, take the answer you think is correct. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Wenn Sie sich nicht sicher sind, nehmen Sie die Antwort, die Sie für richtig halten. </t>
-  </si>
-  <si>
-    <t>In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. \\ 
-Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Zuerst wirst du Beispiele hören und dann ein paar Übungsaufgaben machen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bitte drücken Sie die Starttaste, um die Musik zu starten. \\\\ In diesem Beispiel ist das Zielsintrument (Piano) in der Mixtur zu hören.
-</t>
   </si>
   <si>
     <t xml:space="preserve">Bitte drücken Sie die Starttaste, um die Musik zu starten. \\\\ In diesem Beispiel ist das Zielsintrument (Hauptgesang) nicht in der Mixtur zu hören.
@@ -236,60 +197,108 @@
     <t xml:space="preserve">Please press the start button to launch the music. \\\\ Here, the target instrument (lead voice) does not play in the mixture. </t>
   </si>
   <si>
-    <t>&lt;h4&gt;Welcome to the test for musical scene analysis (MSA)&lt;/h4&gt;  In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (lead voice, bass, guitar or piano) plays, in the second part a mixture of several instruments (mixture) plays. 
-Your task is to decide whether the single target instrument played in the mixture of instruments. \\
-Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture".\\ First, you’ll hear some examples and do a few practice questions.</t>
+    <t>PRACTICE3</t>
+  </si>
+  <si>
+    <t>falsch.</t>
+  </si>
+  <si>
+    <t>richtig!</t>
+  </si>
+  <si>
+    <t>incorrect.</t>
+  </si>
+  <si>
+    <t>correct!</t>
+  </si>
+  <si>
+    <t>PRACTICE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The anwser was **{{feedback}}** \\ Press ‘Go back’ to read the instructions and do the practice questions again, or press ‘Continue’ to continue to the main test. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please press the start button to launch the music. \\\\ Here, the target instrument (lead voice) plays in the mixture. </t>
   </si>
   <si>
     <t xml:space="preserve">In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (lead voice, bass, guitar or piano) plays, in the second part a mixture of several instruments (mixture) plays. 
 Your task is to decide whether the single target instrument played in the mixture of instruments. \\
-Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture".\\ First, you’ll hear some examples and do a few practice questions.
+Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture".\\ First, you’ll hear some examples and do a few practice questions.
 </t>
   </si>
   <si>
-    <t>PRACTICE3</t>
-  </si>
-  <si>
-    <t>falsch.</t>
-  </si>
-  <si>
-    <t>richtig!</t>
-  </si>
-  <si>
-    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 2** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
-  </si>
-  <si>
-    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 4** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
-  </si>
-  <si>
-    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 3** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
-  </si>
-  <si>
-    <t>Die Antwort war  **{{feedback}}** \\ Klicke auf 'Zurück', um die Anweisungen erneut zu lesen und die Beispiele erneut zu versuchen, oder klicke auf 'Weiter', um zum  Haupttest zu gelangen.</t>
-  </si>
-  <si>
-    <t>The anwser was  **{{feedback}}** \\ **Practice question 2** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
-  </si>
-  <si>
-    <t>The anwser was **{{feedback}}** \\ **Practice question 3** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
-  </si>
-  <si>
-    <t>The anwser was **{{feedback}}** \\ **Practice question 4** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
-  </si>
-  <si>
-    <t>incorrect.</t>
-  </si>
-  <si>
-    <t>correct!</t>
-  </si>
-  <si>
-    <t>PRACTICE4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The anwser was **{{feedback}}** \\ Press ‘Go back’ to read the instructions and do the practice questions again, or press ‘Continue’ to continue to the main test. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please press the start button to launch the music. \\\\ Here, the target instrument (lead voice) plays in the mixture. </t>
+    <t xml:space="preserve">Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture.\\ If you are not sure, take the answer you think is correct. </t>
+  </si>
+  <si>
+    <t>**Practice question 1** \\ Please listen to the following clip and and decide, whether the target plays in the mixture.\\ Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>The anwser was  **{{feedback}}** \\ **Practice question 2** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>The anwser was **{{feedback}}** \\ **Practice question 3** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>The anwser was **{{feedback}}** \\ **Practice question 4** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. \\ 
+Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "No" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Zuerst wirst du Beispiele hören und dann ein paar Übungsaufgaben machen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "No" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Wenn Sie sich nicht sicher sind, nehmen Sie die Antwort, die Sie für richtig halten. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitte drücken Sie die Starttaste, um die Musik zu starten. \\\\ In diesem Beispiel ist das Zielsintrument (Hauptgesang) in der Mixtur zu hören.
+</t>
+  </si>
+  <si>
+    <t>**Übungsfrage 1** \\ Bitte hören Sie sich den folgenden Clip an und entscheiden Sie, ob das Zielinstrument in der Instrumentenmixtur spielte.\\ Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 2** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 3** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t>Die Antwort war **{{feedback}}** \\ **Übungsfrage 4** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Willkommen zum Test zur Musikalischen Szenenanalysen (MSA)&lt;/h4&gt; In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. \\ 
+Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Zuerst wirst du Beispiele hören und dann ein paar Übungsaufgaben machen.</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Welcome to the test for musical scene analysis (MSA)&lt;/h4&gt;  In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (lead voice, bass, guitar or piano) plays, in the second part a mixture of several instruments (mixture) plays. \\
+&lt;strong&gt; Your task is to decide whether the single target instrument played in the mixture of instruments. &lt;/strong&gt; \\
+Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture".\\ First, you’ll hear some examples and do a few practice questions.</t>
+  </si>
+  <si>
+    <t>FINAL_P</t>
+  </si>
+  <si>
+    <t>Sie haben den Test zur musikalischen Szenenanalyse erfolgreich beendet. Ihre Daten wurden gespeichert. \\ &lt;strong&gt; Sie können den Browser jetzt schließen. &lt;/strong&gt;</t>
+  </si>
+  <si>
+    <t>You have successfully completed the musical scene analysis test. Your data has been saved. \\ &lt;strong&gt;You can now close the browser. &lt;/strong&gt;</t>
+  </si>
+  <si>
+    <t>Die Antwort war  **{{feedback}}** \\ Klicken Sie auf 'Zurück', um die Anweisungen erneut zu lesen und die Beispiele erneut zu versuchen, oder klicke auf 'Weiter', um zum  Haupttest zu gelangen.</t>
+  </si>
+  <si>
+    <t>Ihr Browser unterstützt kein Audio. Dieser Test funktioniert nicht ohne Audio! Probieren Sie es bitte mit einem anderen Browser (bspw. Google Chrome).</t>
+  </si>
+  <si>
+    <t>Die ID ist leider ungültig. Bitte versuchen Sie es noch mal.</t>
+  </si>
+  <si>
+    <t>Sie haben den Test zur musikalischen Szenenanalyse erfolgreich beendet.</t>
+  </si>
+  <si>
+    <t>Sie haben {{num_correct}} von {{num_question}} Fragen richtig beantwortet.</t>
+  </si>
+  <si>
+    <t>Ihr Testergebnis</t>
   </si>
 </sst>
 </file>
@@ -717,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -741,10 +750,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -752,10 +761,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -766,7 +775,7 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -774,10 +783,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -785,10 +794,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -799,7 +808,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -810,7 +819,7 @@
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -818,10 +827,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -832,7 +841,7 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -840,10 +849,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -851,10 +860,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -862,10 +871,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -873,10 +882,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -884,10 +893,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -895,10 +904,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -906,142 +915,153 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="120" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>77</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>58</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the adaptive MSA and include a beautiful graphical scoring feedback for participants.
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Dropbox\Uni Oldenburg\#3 - RStudio dateien\#4 - MSAT - main test R script\MSA\data_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83471C14-FC0E-43ED-9944-5FC57D82CA79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42F5A3B-84F3-4B0D-A87D-2C22A833143F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1890" windowWidth="38640" windowHeight="20865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1680" windowWidth="38640" windowHeight="20595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EDT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>key</t>
   </si>
@@ -118,16 +118,7 @@
     <t>You answered {{num_correct}} out of {{num_question}} questions correctly.</t>
   </si>
   <si>
-    <t>Your score</t>
-  </si>
-  <si>
     <t>Score</t>
-  </si>
-  <si>
-    <t>Musikalische Szenenanalyse Test</t>
-  </si>
-  <si>
-    <t>Musical Scene Analysis Test</t>
   </si>
   <si>
     <t>You have completed the Musical Scene Analysis test.</t>
@@ -298,17 +289,68 @@
     <t>Sie haben {{num_correct}} von {{num_question}} Fragen richtig beantwortet.</t>
   </si>
   <si>
-    <t>Ihr Testergebnis</t>
+    <t>This score indicates that you perform better than</t>
+  </si>
+  <si>
+    <t>percent of the test takers</t>
+  </si>
+  <si>
+    <t>Probability Density (%)</t>
+  </si>
+  <si>
+    <t>FEEDBACK_Y</t>
+  </si>
+  <si>
+    <t>FEEDBACK_X1</t>
+  </si>
+  <si>
+    <t>FEEDBACK_X2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ihr MSA Testergebnis: </t>
+  </si>
+  <si>
+    <t>Your MSA score:</t>
+  </si>
+  <si>
+    <t>Musikalische Szenenanalyse (MSA) Test</t>
+  </si>
+  <si>
+    <t>Musical Scene Analysis (MSA) Test</t>
+  </si>
+  <si>
+    <t>Diese Bewertung zeigt an, dass Sie besser abschneiden als</t>
+  </si>
+  <si>
+    <t>Prozent der Testpersonen</t>
+  </si>
+  <si>
+    <t>Wahrscheinlichkeitsdichte (%)</t>
+  </si>
+  <si>
+    <t>Verteilung</t>
+  </si>
+  <si>
+    <t>Distribution</t>
+  </si>
+  <si>
+    <t>FEEDBACK_TITLE1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -407,7 +449,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -726,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -750,10 +792,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -761,10 +803,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -783,10 +825,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -794,10 +836,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -827,10 +869,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -849,7 +891,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
         <v>29</v>
@@ -871,10 +913,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -882,10 +924,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -893,7 +935,7 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -901,170 +943,218 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="B19" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="120" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="B20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B21" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C29" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>82</v>
+        <v>17</v>
+      </c>
+      <c r="B30" t="s">
+        <v>92</v>
       </c>
       <c r="C30" t="s">
-        <v>83</v>
-      </c>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="8"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D33" s="8"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="8"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
changes to default MSA command
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BA6B01-75F8-4C6F-AF60-1E38FC074201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F28DB65-86C9-421E-9D4F-268167D362D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1680" windowWidth="38640" windowHeight="20595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="405" windowWidth="29040" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSA" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="136">
   <si>
     <t>key</t>
   </si>
@@ -463,6 +463,9 @@
     <t xml:space="preserve">In this task, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (lead voice, bass, guitar or piano) plays, in the second part a mixture of several instruments (mixture) plays. \\ 
 &lt;strong&gt; Your task is to decide whether the single target instrument played in the mixture of instruments. &lt;/strong&gt; \\ By clicking on "Continue", the test begins and your responses will be saved.
 </t>
+  </si>
+  <si>
+    <t>FR</t>
   </si>
 </sst>
 </file>
@@ -584,7 +587,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -903,7 +906,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -913,7 +916,7 @@
     <col min="5" max="6" width="123.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -926,8 +929,11 @@
       <c r="D1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -941,7 +947,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -955,7 +961,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -969,7 +975,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -983,7 +989,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -997,7 +1003,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1011,7 +1017,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1025,7 +1031,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1039,7 +1045,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1053,7 +1059,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1067,7 +1073,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1081,7 +1087,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -1095,7 +1101,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1109,7 +1115,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1123,7 +1129,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
add example experiment code & FR langauge
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F28DB65-86C9-421E-9D4F-268167D362D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87E7369-C2AF-4543-962A-D5E1F15E7D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="405" windowWidth="29040" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSA" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="183">
   <si>
     <t>key</t>
   </si>
@@ -467,12 +467,306 @@
   <si>
     <t>FR</t>
   </si>
+  <si>
+    <t>INSTRUCTIONS_LONG</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Welcome to the Musical Scene Analysis (MSA) Test&lt;/h4&gt;
+    &lt;p&gt;In this test, you will be presented with a series of music excerpts. Each excerpt is structured as follows:&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Initial Music Segment (8 seconds):&lt;/strong&gt; A song will play for 8 seconds. This is the initial music segment.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Pause (1 second):&lt;/strong&gt; After the initial music segment, there will be a 1-second pause.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Target Instrument Segment:&lt;/strong&gt; Following the pause, a single instrument (either a lead voice, bass, guitar, or piano) will play. This is the target instrument.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Pause (1 second):&lt;/strong&gt; After the target instrument segment, there will be another 1-second pause.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;5. Mixture Segment (2 seconds):&lt;/strong&gt; Finally, a mixture of several instruments will play for 2 seconds. This is the mixture segment. The target instrument may or may not be included in this mixture.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Your task is to determine whether the target instrument that played after the first pause is included in the final mixture segment.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Please listen carefully to each segment and make your decision based on the sounds you hear. Good luck!&lt;/p&gt;
+    &lt;p&gt;Before the data collection begins, you will have the opportunity to hear some examples and do some practice trials. This will help you understand the task better and prepare you for the actual test.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Segment Musical Initial (8 secondes) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Une chanson jouera pendant 8 secondes. C'est le segment musical initial.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. Pause (1 seconde) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Après le segment musical initial, il y aura une pause de 1 seconde.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. Segment de l'Instrument Cible :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Suite à la pause, un seul instrument (soit une voix principale, une basse, une guitare, ou un piano) jouera. C'est l'instrument cible.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Pause (1 seconde) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Après le segment de l'instrument cible, il y aura une autre pause de 1 seconde.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5. Segment de Mélange (2 secondes) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.</t>
+    </r>
+  </si>
+  <si>
+    <t>Votre tâche est de déterminer si l'instrument cible qui a joué après la première pause est inclus dans le segment de mélange final.</t>
+  </si>
+  <si>
+    <t>Veuillez écouter attentivement chaque segment et prendre votre décision en fonction des sons que vous entendez. Bonne chance!</t>
+  </si>
+  <si>
+    <t>Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.</t>
+  </si>
+  <si>
+    <t>&lt;body&gt;
+    &lt;h4&gt;Bienvenue au test d'Analyse de Scène Musicale (ASM)&lt;/h4&gt;
+    &lt;p&gt;Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Segment Musical Initial (8 secondes) :&lt;/strong&gt; Une chanson jouera pendant 8 secondes. C'est le segment musical initial.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Pause (1 seconde) :&lt;/strong&gt; Après le segment musical initial, il y aura une pause de 1 seconde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Segment de l'Instrument Cible :&lt;/strong&gt; Suite à la pause, un seul instrument (soit une voix principale, une basse, une guitare, ou un piano) jouera. C'est l'instrument cible.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Pause (1 seconde) :&lt;/strong&gt; Après le segment de l'instrument cible, il y aura une autre pause de 1 seconde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;5. Segment de Mélange (2 secondes) :&lt;/strong&gt; Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Votre tâche est de déterminer si l'instrument cible qui a joué après la première pause est inclus dans le segment de mélange final.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Veuillez écouter attentivement chaque segment et prendre votre décision en fonction des sons que vous entendez. Bonne chance!&lt;/p&gt;
+    &lt;p&gt;Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.&lt;/p&gt;
+&lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>&lt;body&gt;
+    &lt;h4&gt;Willkommen zum Test für Musikalische Szenenanalyse (MSA)&lt;/h4&gt;
+    &lt;p&gt;In diesem Test werden Ihnen eine Reihe von Musikausschnitten präsentiert. Jeder Ausschnitt ist wie folgt strukturiert:&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Pause (1 Sekunde):&lt;/strong&gt; Nach dem anfänglichen Musiksegment gibt es eine Pause von 1 Sekunde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Nach der Pause spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine weitere Pause von 1 Sekunde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;5. Mischsegment (2 Sekunden):&lt;/strong&gt; Schließlich spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist das Mischsegment. Das Zielinstrument kann in dieser Mischung enthalten sein oder auch nicht.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Ihre Aufgabe besteht darin zu bestimmen, ob das Zielinstrument, das nach der ersten Pause gespielt hat, im abschließenden Mischsegment enthalten ist.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Bitte hören Sie jedes Segment sorgfältig an und treffen Sie Ihre Entscheidung auf der Grundlage der Geräusche, die Sie hören. Viel Glück!&lt;/p&gt;
+    &lt;p&gt;Bevor die Datenerfassung beginnt, haben Sie die Möglichkeit, einige Beispiele zu hören und einige Übungsdurchläufe zu machen. Dies wird Ihnen helfen, die Aufgabe besser zu verstehen und sich auf den eigentlichen Test vorzubereiten.&lt;/p&gt;
+&lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>&lt;body&gt;
+    &lt;h4&gt;Willkommen zum Musikalische Szenenanalyse (MSA) Test&lt;/h4&gt;
+    &lt;p&gt;In diesem Test bekommst du eine Reihe von Musikausschnitten vorgespielt. Jeder Ausschnitt ist so aufgebaut:&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Anfangs Musikstück (8 Sekunden):&lt;/strong&gt; Ein Lied spielt für 8 Sekunden. Das ist das Anfangs Musikstück.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Anfangs Musikstück gibt's eine Pause von 1 Sekunde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Zielinstrument Abschnitt:&lt;/strong&gt; Nach der Pause spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Das ist das Zielinstrument.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrument Abschnitt gibt's nochmal eine Pause von 1 Sekunde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;5. Mischung Abschnitt (2 Sekunden):&lt;/strong&gt; Zum Schluss spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Das ist der Mischung Abschnitt. Das Zielinstrument könnte in dieser Mischung sein, oder auch nicht.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Deine Aufgabe ist es zu entscheiden, ob das Zielinstrument, das nach der ersten Pause gespielt hat, in der abschließenden Mischung ist.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Hör dir jedes Segment genau an und triff deine Entscheidung basierend auf den Klängen, die du hörst. Viel Glück!&lt;/p&gt;
+    &lt;p&gt;Bevor wir mit der Datensammlung anfangen, hast du die Möglichkeit, ein paar Beispiele zu hören und ein paar Übungsdurchläufe zu machen. Das hilft dir, die Aufgabe besser zu verstehen und dich auf den eigentlichen Test vorzubereiten.&lt;/p&gt;
+&lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>Bienvenu pour ce test d'analyse de scènes musicales</t>
+  </si>
+  <si>
+    <t>Des extraits musicaux vont être présentés pour ce test. Chaque extrait est en deux parties. Un extrait avec un instrument seul (voix, basse, guitare ou piano) est présenté  dans un premier temps, puis un mélange avec plusieurs instruments (Mix). \\ &lt;strong&gt; Votre tâche est de décider, si l'instrument présenté seul est aussi présent dans le mix avec plusieurs instruments. &lt;/strong&gt;\\ Le test commence et vos réponses sont enregistrées quand vous cliquez sur "suivant".</t>
+  </si>
+  <si>
+    <t>Question {{num_question}} sur {{test_length}}</t>
+  </si>
+  <si>
+    <t>Votre navigateur ne supporte pas l'audio. Ce test ne fonctionne pas sans audio! Essayez avec un autre navigateur (Chrome par expl.)</t>
+  </si>
+  <si>
+    <t>Cliquez sur "Oui, l'instrument seul est dans le mix" ou sur "Non, l'instrument seul n'est pas dans le mix".\\ Choisissez la réponse qui vous paraît être la plus probable si vous hésitez.</t>
+  </si>
+  <si>
+    <t>Choisissez une option s'il vous plaît</t>
+  </si>
+  <si>
+    <t>Félicitations !</t>
+  </si>
+  <si>
+    <t>Vous avez reconnu **{{accuracy}} %** des instruments de musique.</t>
+  </si>
+  <si>
+    <t>Entrez un identifiant</t>
+  </si>
+  <si>
+    <t>L'identifiant n'est pas valide. Essayez à nouveau.</t>
+  </si>
+  <si>
+    <t>Suivant</t>
+  </si>
+  <si>
+    <t>Vous avez terminé avec succès le test d'analyse des scènes musicales.</t>
+  </si>
+  <si>
+    <t>Test d'analyse des scènes musicales (MSA)</t>
+  </si>
+  <si>
+    <t>Vous avez répondu correctement à  {{num_correct}} sur {{num_question}} questions.</t>
+  </si>
+  <si>
+    <t>Scores</t>
+  </si>
+  <si>
+    <t>Revenir en arrière</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Bienvenu au test d'analyse des scènes musicales (MSA)&lt;/h4&gt;Des extraits musicaux vont être présentés pour ce test. Chaque extrait est en deux parties. Un extrait avec un instrument seul (voix, basse, guitare ou piano) est présenté  dans un premier temps, puis un mélange avec plusieurs instruments (Mix). \\
+Votre tâche est de décider, si l'instrument seul est présent dans le mix avec plusieurs instruments. &lt;/strong&gt;\\ 
+Vous avez la possibilité d'écouter quelques extraits et de vous entraîner avant de commencer le test.</t>
+  </si>
+  <si>
+    <t>Vous avez la possibilité d'écouter quelques exemples. &lt;strong&gt;  Appuyez sur "Start" pour commencer à écouter.&lt;/strong&gt;  \\\\ L'instrument cible (voix) est présent dans le mix pour cet exemple.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;strong&gt; Appuyez sur "Start" pour commencer à écouter.&lt;/strong&gt;  \\\\ L'instrument cible (voix) n'est pas présent dans le mix pour cet exemple.
+</t>
+  </si>
+  <si>
+    <t>**Exemple 1** \\ Ecoutez l'extrait musical suivant et indiquez si l'instrument cible est présent dans le mix.\\ Cliquez sur "Oui, l'instrument cible est présent dans le mix" ou "Non, l'instrument cible n'est pas dans le mix".</t>
+  </si>
+  <si>
+    <t>La réponse est **{{feedback}}** &lt;p&gt;&amp;nbsp;&lt;/p&gt; \\\\ **Exemple 2** \\Ecoutez l'extrait musical suivant et indiquez si l'instrument cible est présent dans le mix.\\ Cliquez sur "Oui, l'instrument cible est présent dans le mix" ou "Non, l'instrument cible n'est pas dans le mix".</t>
+  </si>
+  <si>
+    <t>La réponse est **{{feedback}}** &lt;p&gt;&amp;nbsp;&lt;/p&gt; \\\\ **Exemple 3** \\Ecoutez l'extrait musical suivant et indiquez si l'instrument cible est présent dans le mix.\\ Cliquez sur "Oui, l'instrument cible est présent dans le mix" ou "Non, l'instrument cible n'est pas dans le mix".</t>
+  </si>
+  <si>
+    <t>La réponse est **{{feedback}}** &lt;p&gt;&amp;nbsp;&lt;/p&gt; \\\\ **Exemple 4** \\Ecoutez l'extrait musical suivant et indiquez si l'instrument cible est présent dans le mix.\\ Cliquez sur "Oui, l'instrument cible est présent dans le mix" ou "Non, l'instrument cible n'est pas dans le mix".</t>
+  </si>
+  <si>
+    <t>La réponse était  **{{feedback}}**&lt;p&gt;&amp;nbsp;&lt;/p&gt;  \\\\ Cliquez sur "revenir en arrière", pour lire à nouveau les instructions et vous entraîner avec les exemples ou cliquez sur "suivant" pour commencer avec le test principal.</t>
+  </si>
+  <si>
+    <t>faux</t>
+  </si>
+  <si>
+    <t>Nous commençons maintenant avec le test principal où vos réponses sont comptabilisées. \\ Vous ne rceverez plus de retour à partir de maintenant. Bon courage !</t>
+  </si>
+  <si>
+    <t>Vous avec terminé avec le test d'analyse de scènes musicales avec succès. \\ &lt;strong&gt; Vous pouvez fermer votre navigateur internet. &lt;/strong&gt;</t>
+  </si>
+  <si>
+    <t>Votre résultat du MSA:</t>
+  </si>
+  <si>
+    <t>Cette analyse indique que vos résultats sont meilleurs que</t>
+  </si>
+  <si>
+    <t>pourcent des participants au test</t>
+  </si>
+  <si>
+    <t>densité de probabilité (%)</t>
+  </si>
+  <si>
+    <t>Oui - l'instrument cible est dans le mix</t>
+  </si>
+  <si>
+    <t>Non - l'instrument cible n'est pas dans le mix</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -489,6 +783,28 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -514,20 +830,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -587,7 +906,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -906,13 +1225,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
     <col min="2" max="2" width="123.7109375" customWidth="1"/>
-    <col min="3" max="3" width="150.5703125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="150.5703125" customWidth="1"/>
+    <col min="3" max="4" width="150.5703125" customWidth="1"/>
     <col min="5" max="6" width="123.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -923,7 +1241,7 @@
       <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
@@ -940,25 +1258,31 @@
       <c r="B2" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" t="s">
         <v>49</v>
       </c>
       <c r="D2" t="s">
         <v>49</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="1" t="s">
         <v>133</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -968,11 +1292,14 @@
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" t="s">
         <v>19</v>
       </c>
       <c r="D4" t="s">
         <v>19</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -982,11 +1309,14 @@
       <c r="B5" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" t="s">
         <v>106</v>
       </c>
       <c r="D5" t="s">
         <v>60</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -996,11 +1326,14 @@
       <c r="B6" t="s">
         <v>127</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" t="s">
         <v>107</v>
       </c>
       <c r="D6" t="s">
         <v>95</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1010,11 +1343,14 @@
       <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1024,11 +1360,14 @@
       <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" t="s">
         <v>21</v>
       </c>
       <c r="D8" t="s">
         <v>21</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1038,11 +1377,14 @@
       <c r="B9" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" t="s">
         <v>33</v>
       </c>
       <c r="D9" t="s">
         <v>108</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1052,11 +1394,14 @@
       <c r="B10" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" t="s">
         <v>109</v>
       </c>
       <c r="D10" t="s">
         <v>96</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1066,11 +1411,14 @@
       <c r="B11" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" t="s">
         <v>110</v>
       </c>
       <c r="D11" t="s">
         <v>61</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1080,11 +1428,14 @@
       <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1094,11 +1445,14 @@
       <c r="B13" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" t="s">
         <v>111</v>
       </c>
       <c r="D13" t="s">
         <v>62</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1108,11 +1462,14 @@
       <c r="B14" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" t="s">
         <v>72</v>
       </c>
       <c r="D14" t="s">
         <v>72</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1122,11 +1479,14 @@
       <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" t="s">
         <v>112</v>
       </c>
       <c r="D15" t="s">
         <v>63</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1136,333 +1496,467 @@
       <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" t="s">
         <v>23</v>
       </c>
       <c r="D16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="E16" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="E17" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="E18" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="E19" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="E20" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="E21" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" t="s">
         <v>84</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="E22" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" t="s">
         <v>98</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="E23" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" t="s">
         <v>128</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="E24" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" t="s">
         <v>129</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" t="s">
         <v>117</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="E25" s="6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" t="s">
         <v>130</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" t="s">
         <v>118</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="E26" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" t="s">
         <v>131</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" t="s">
         <v>119</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="E27" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" t="s">
         <v>104</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" t="s">
         <v>120</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+      <c r="E28" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" t="s">
         <v>52</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+      <c r="E29" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" t="s">
         <v>53</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+      <c r="E30" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>46</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" t="s">
         <v>123</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E31" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>57</v>
       </c>
       <c r="B32" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" t="s">
         <v>124</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" s="6" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>17</v>
       </c>
       <c r="B33" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" t="s">
         <v>125</v>
       </c>
       <c r="D33" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="E33" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>79</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" t="s">
         <v>77</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" t="s">
         <v>126</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="E35" s="6" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
+      <c r="E36" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>67</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" t="s">
         <v>66</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>88</v>
       </c>
       <c r="B38" t="s">
         <v>91</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" t="s">
         <v>90</v>
       </c>
       <c r="D38" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
+      <c r="E38" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>89</v>
       </c>
       <c r="B39" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" t="s">
         <v>93</v>
       </c>
       <c r="D39" t="s">
         <v>93</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding a long version of the MSA for haring-impaired and CI users
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87E7369-C2AF-4543-962A-D5E1F15E7D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA39A61-7773-4BD9-B44C-93A9C1474C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-2205" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSA" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="190">
   <si>
     <t>key</t>
   </si>
@@ -761,12 +761,33 @@
   <si>
     <t>Non - l'instrument cible n'est pas dans le mix</t>
   </si>
+  <si>
+    <t>INSTRUCTIONS_PIC_LONG</t>
+  </si>
+  <si>
+    <t>INSTRUCTIONS_PIC_SHORT</t>
+  </si>
+  <si>
+    <t>https://www.testable.org/experiment/4346/515133/stimuli/FR_long.png</t>
+  </si>
+  <si>
+    <t>https://www.testable.org/experiment/4346/515133/stimuli/DE_long.png</t>
+  </si>
+  <si>
+    <t>https://www.testable.org/experiment/4346/515133/stimuli/EN_long.png</t>
+  </si>
+  <si>
+    <t>https://www.testable.org/experiment/4346/515133/stimuli/EN_short.png</t>
+  </si>
+  <si>
+    <t>https://www.testable.org/experiment/4346/515133/stimuli/DE_short.png</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -809,6 +830,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -827,10 +856,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -843,15 +873,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1225,7 +1252,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -1264,7 +1291,7 @@
       <c r="D2" t="s">
         <v>49</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" t="s">
         <v>150</v>
       </c>
     </row>
@@ -1281,7 +1308,7 @@
       <c r="D3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="1" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1298,7 +1325,7 @@
       <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1315,7 +1342,7 @@
       <c r="D5" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1332,7 +1359,7 @@
       <c r="D6" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1349,7 +1376,7 @@
       <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1366,7 +1393,7 @@
       <c r="D8" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" t="s">
         <v>156</v>
       </c>
     </row>
@@ -1383,7 +1410,7 @@
       <c r="D9" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" t="s">
         <v>157</v>
       </c>
     </row>
@@ -1400,7 +1427,7 @@
       <c r="D10" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1417,7 +1444,7 @@
       <c r="D11" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" t="s">
         <v>159</v>
       </c>
     </row>
@@ -1434,7 +1461,7 @@
       <c r="D12" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1451,7 +1478,7 @@
       <c r="D13" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" t="s">
         <v>161</v>
       </c>
     </row>
@@ -1468,7 +1495,7 @@
       <c r="D14" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" t="s">
         <v>162</v>
       </c>
     </row>
@@ -1485,7 +1512,7 @@
       <c r="D15" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" t="s">
         <v>163</v>
       </c>
     </row>
@@ -1502,7 +1529,7 @@
       <c r="D16" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1519,7 +1546,7 @@
       <c r="D17" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" t="s">
         <v>165</v>
       </c>
     </row>
@@ -1536,7 +1563,7 @@
       <c r="D18" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="1" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1544,7 +1571,7 @@
       <c r="A19" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1553,7 +1580,7 @@
       <c r="D19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1561,7 +1588,7 @@
       <c r="A20" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="6" t="s">
         <v>83</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1570,7 +1597,7 @@
       <c r="D20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="2" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1587,382 +1614,426 @@
       <c r="D21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>184</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>39</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B24" t="s">
         <v>84</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E24" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>40</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B25" t="s">
         <v>98</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E25" s="1" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" t="s">
-        <v>116</v>
-      </c>
-      <c r="D24" t="s">
-        <v>94</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" t="s">
-        <v>129</v>
-      </c>
-      <c r="C25" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" t="s">
-        <v>101</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="B26" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D26" t="s">
-        <v>102</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>171</v>
+        <v>94</v>
+      </c>
+      <c r="E26" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D27" t="s">
-        <v>103</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>172</v>
+        <v>101</v>
+      </c>
+      <c r="E27" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B28" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>173</v>
+        <v>102</v>
+      </c>
+      <c r="E28" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>54</v>
+        <v>131</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>119</v>
       </c>
       <c r="D29" t="s">
-        <v>52</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>174</v>
+        <v>103</v>
+      </c>
+      <c r="E29" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="D30" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>55</v>
+        <v>121</v>
+      </c>
+      <c r="E30" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>52</v>
       </c>
       <c r="D31" t="s">
-        <v>122</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>175</v>
+        <v>52</v>
+      </c>
+      <c r="E31" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
-        <v>58</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>176</v>
+        <v>53</v>
+      </c>
+      <c r="E32" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B33" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D33" t="s">
-        <v>70</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>177</v>
+        <v>122</v>
+      </c>
+      <c r="E33" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="D34" t="s">
-        <v>77</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>78</v>
+        <v>58</v>
+      </c>
+      <c r="E34" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="B35" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D35" t="s">
-        <v>74</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>178</v>
+        <v>70</v>
+      </c>
+      <c r="E35" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D36" t="s">
-        <v>75</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>179</v>
+        <v>77</v>
+      </c>
+      <c r="E36" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="D37" t="s">
-        <v>76</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>180</v>
+        <v>74</v>
+      </c>
+      <c r="E37" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>181</v>
+        <v>75</v>
+      </c>
+      <c r="E38" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>89</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B41" t="s">
         <v>92</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C41" t="s">
         <v>93</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D41" t="s">
         <v>93</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E41" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="42" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>136</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E42" s="3" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="3" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E44" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E45" s="4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E46" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="4" t="s">
         <v>144</v>
-      </c>
-    </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E51" s="3" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E53" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="3" t="s">
         <v>146</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B19" r:id="rId1" xr:uid="{72C03BFD-2C2C-4707-8455-9A3685430207}"/>
+    <hyperlink ref="B20" r:id="rId2" xr:uid="{2C3AE3AC-D225-4C7C-B120-2FAFB3C93CA5}"/>
+    <hyperlink ref="B22" r:id="rId3" xr:uid="{189D53A6-5BED-420A-AA21-B45B532602A1}"/>
+    <hyperlink ref="C22" r:id="rId4" xr:uid="{6D9380BD-D329-4F17-AB89-CEAFD850206A}"/>
+    <hyperlink ref="D22" r:id="rId5" xr:uid="{60357076-1E21-4A27-917E-9EC72998F0AB}"/>
+    <hyperlink ref="C23" r:id="rId6" xr:uid="{8CC740FC-ED34-4EA6-BEC1-9755BB240220}"/>
+    <hyperlink ref="D23" r:id="rId7" xr:uid="{EB036BEC-9ACC-4F6B-9B4A-58C5412FBB8A}"/>
+    <hyperlink ref="E23" r:id="rId8" xr:uid="{74D081F7-7134-44DA-8150-E8559DD4009D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix some bugs and add proper instructions
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA39A61-7773-4BD9-B44C-93A9C1474C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5393E2D5-94D7-4094-A27B-260F939D49AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2205" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="194">
   <si>
     <t>key</t>
   </si>
@@ -660,9 +660,6 @@
 &lt;/body&gt;</t>
   </si>
   <si>
-    <t>Bienvenu pour ce test d'analyse de scènes musicales</t>
-  </si>
-  <si>
     <t>Des extraits musicaux vont être présentés pour ce test. Chaque extrait est en deux parties. Un extrait avec un instrument seul (voix, basse, guitare ou piano) est présenté  dans un premier temps, puis un mélange avec plusieurs instruments (Mix). \\ &lt;strong&gt; Votre tâche est de décider, si l'instrument présenté seul est aussi présent dans le mix avec plusieurs instruments. &lt;/strong&gt;\\ Le test commence et vos réponses sont enregistrées quand vous cliquez sur "suivant".</t>
   </si>
   <si>
@@ -781,6 +778,21 @@
   </si>
   <si>
     <t>https://www.testable.org/experiment/4346/515133/stimuli/DE_short.png</t>
+  </si>
+  <si>
+    <t>Welcome to the test for musical scene analysis (MSA-L)</t>
+  </si>
+  <si>
+    <t>Willkommen zum Test zur Musikalischen Szenenanalysen (MSA-L)</t>
+  </si>
+  <si>
+    <t>Bienvenu pour ce test d'analyse de scènes musicales (MSA-L)</t>
+  </si>
+  <si>
+    <t>Bienvenu pour ce test d'analyse de scènes musicales (MSA)</t>
+  </si>
+  <si>
+    <t>WELCOME_LONG</t>
   </si>
 </sst>
 </file>
@@ -900,13 +912,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>203200</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>23906</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1252,7 +1264,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -1292,745 +1304,762 @@
         <v>49</v>
       </c>
       <c r="E2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>95</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
+        <v>111</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="E15" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="E16" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D18" t="s">
         <v>36</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>165</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>80</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>183</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>186</v>
+        <v>86</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>185</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>182</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B23" s="2" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>183</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" t="s">
-        <v>84</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>167</v>
+      <c r="D24" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>40</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" t="s">
-        <v>128</v>
-      </c>
-      <c r="C26" t="s">
-        <v>116</v>
-      </c>
-      <c r="D26" t="s">
-        <v>94</v>
-      </c>
-      <c r="E26" t="s">
-        <v>169</v>
+      <c r="E26" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="E30" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B31" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>120</v>
       </c>
       <c r="D31" t="s">
-        <v>52</v>
+        <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E32" t="s">
-        <v>55</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>46</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>47</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>123</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>122</v>
       </c>
-      <c r="E33" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" t="s">
-        <v>124</v>
-      </c>
-      <c r="D34" t="s">
-        <v>58</v>
-      </c>
       <c r="E34" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="B35" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C35" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D35" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>125</v>
       </c>
       <c r="D36" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="C37" t="s">
-        <v>126</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E37" t="s">
-        <v>178</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C38" t="s">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="D38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E39" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E40" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" t="s">
+        <v>90</v>
+      </c>
+      <c r="D41" t="s">
+        <v>90</v>
+      </c>
+      <c r="E41" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>89</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>92</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C42" t="s">
         <v>93</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D42" t="s">
         <v>93</v>
       </c>
-      <c r="E41" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="E42" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>136</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E44" s="3" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="3" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E46" s="4" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E50" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E51" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="4" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E53" s="3" t="s">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="3" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E55" s="3" t="s">
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="3" t="s">
         <v>146</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B19" r:id="rId1" xr:uid="{72C03BFD-2C2C-4707-8455-9A3685430207}"/>
-    <hyperlink ref="B20" r:id="rId2" xr:uid="{2C3AE3AC-D225-4C7C-B120-2FAFB3C93CA5}"/>
-    <hyperlink ref="B22" r:id="rId3" xr:uid="{189D53A6-5BED-420A-AA21-B45B532602A1}"/>
-    <hyperlink ref="C22" r:id="rId4" xr:uid="{6D9380BD-D329-4F17-AB89-CEAFD850206A}"/>
-    <hyperlink ref="D22" r:id="rId5" xr:uid="{60357076-1E21-4A27-917E-9EC72998F0AB}"/>
-    <hyperlink ref="C23" r:id="rId6" xr:uid="{8CC740FC-ED34-4EA6-BEC1-9755BB240220}"/>
-    <hyperlink ref="D23" r:id="rId7" xr:uid="{EB036BEC-9ACC-4F6B-9B4A-58C5412FBB8A}"/>
-    <hyperlink ref="E23" r:id="rId8" xr:uid="{74D081F7-7134-44DA-8150-E8559DD4009D}"/>
+    <hyperlink ref="B20" r:id="rId1" xr:uid="{72C03BFD-2C2C-4707-8455-9A3685430207}"/>
+    <hyperlink ref="B21" r:id="rId2" xr:uid="{2C3AE3AC-D225-4C7C-B120-2FAFB3C93CA5}"/>
+    <hyperlink ref="B23" r:id="rId3" xr:uid="{189D53A6-5BED-420A-AA21-B45B532602A1}"/>
+    <hyperlink ref="C23" r:id="rId4" xr:uid="{6D9380BD-D329-4F17-AB89-CEAFD850206A}"/>
+    <hyperlink ref="D23" r:id="rId5" xr:uid="{60357076-1E21-4A27-917E-9EC72998F0AB}"/>
+    <hyperlink ref="C24" r:id="rId6" xr:uid="{8CC740FC-ED34-4EA6-BEC1-9755BB240220}"/>
+    <hyperlink ref="D24" r:id="rId7" xr:uid="{EB036BEC-9ACC-4F6B-9B4A-58C5412FBB8A}"/>
+    <hyperlink ref="E24" r:id="rId8" xr:uid="{74D081F7-7134-44DA-8150-E8559DD4009D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>

</xml_diff>

<commit_message>
add / change language settings
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F81F1B-E556-4BDA-99F0-F6E6B516FD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F959174-1392-44F4-9806-D1A7A11B08CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-2205" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSA" sheetId="1" r:id="rId1"/>
@@ -25,12 +25,6 @@
     <t>key</t>
   </si>
   <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
     <t>WELCOME</t>
   </si>
   <si>
@@ -341,9 +335,6 @@
   </si>
   <si>
     <t xml:space="preserve">The anwser was **{{feedback}}** &lt;p&gt;&amp;nbsp;&lt;/p&gt; \\ Press ‘Go back’ to read the instructions and do the practice questions again, or press ‘Continue’ to continue to the main test. </t>
-  </si>
-  <si>
-    <t>DE_F</t>
   </si>
   <si>
     <t>Dein Browser unterstützt kein Audio. Dieser Test funktioniert nicht ohne Audio! Probiere es bitte mit einem anderen Browser (bspw. Google Chrome).</t>
@@ -465,9 +456,6 @@
 </t>
   </si>
   <si>
-    <t>FR</t>
-  </si>
-  <si>
     <t>INSTRUCTIONS_LONG</t>
   </si>
   <si>
@@ -789,6 +777,18 @@
     &lt;/div&gt;
        &lt;p&gt;Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.&lt;/p&gt;
 &lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>fr</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>de_f</t>
   </si>
 </sst>
 </file>
@@ -941,7 +941,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -960,6 +960,57 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="203200" cy="214406"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="dimg_11" descr="coon voor Geverifieerd door de community">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1D497C6-C36C-44D5-82C1-50DE151A7BAB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="30099000" y="1804147"/>
+          <a:ext cx="203200" cy="214406"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1266,7 +1317,7 @@
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
     <col min="2" max="2" width="123.7109375" customWidth="1"/>
     <col min="3" max="4" width="150.5703125" customWidth="1"/>
-    <col min="5" max="6" width="123.7109375" customWidth="1"/>
+    <col min="5" max="5" width="123.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1274,775 +1325,775 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>190</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>193</v>
       </c>
       <c r="E1" t="s">
-        <v>135</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E3" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
-        <v>37</v>
-      </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E18" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="C20" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>174</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>182</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>183</v>
-      </c>
       <c r="C24" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D27" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E27" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C28" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C29" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B30" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E30" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D31" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E31" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D32" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E32" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C33" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33" t="s">
+        <v>51</v>
+      </c>
+      <c r="E33" t="s">
         <v>53</v>
-      </c>
-      <c r="D33" t="s">
-        <v>53</v>
-      </c>
-      <c r="E33" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D34" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E34" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="B35" t="s">
-        <v>59</v>
-      </c>
       <c r="C35" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E35" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E38" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B39" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B40" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D40" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E40" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>86</v>
+      </c>
+      <c r="B41" t="s">
+        <v>89</v>
+      </c>
+      <c r="C41" t="s">
         <v>88</v>
       </c>
-      <c r="B41" t="s">
-        <v>91</v>
-      </c>
-      <c r="C41" t="s">
-        <v>90</v>
-      </c>
       <c r="D41" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E41" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E42" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E45" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E50" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E51" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E52" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E54" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E56" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changing stimuli in long format adding visual support during trials (video content) adding possibility to start MSA with stimuli from local folders
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F959174-1392-44F4-9806-D1A7A11B08CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C2B81B-CB4A-44B2-BA39-2BD290EE87E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2205" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -941,7 +941,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -992,7 +992,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>

</xml_diff>

<commit_message>
changing instruction text of the long version
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C2B81B-CB4A-44B2-BA39-2BD290EE87E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9739EBA-AB9E-49A9-A066-142C57589199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2205" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MSA" sheetId="1" r:id="rId1"/>
@@ -681,20 +681,29 @@
     <t>WELCOME_LONG</t>
   </si>
   <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>fr</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>de_f</t>
+  </si>
+  <si>
     <t>&lt;body&gt;
     &lt;h4&gt;Willkommen zum Test für Musikalische Szenenanalyse (MSA)&lt;/h4&gt;
     &lt;p&gt;In diesem Test wird dir eine Reihe von Musikausschnitten präsentiert. Jeder Ausschnitt ist wie folgt strukturiert:&lt;/p&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment. Bitte höre einfach passiv zu.
     &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;2. Pause (1 Sekunde):&lt;/strong&gt; Nach dem anfänglichen Musiksegment gibt es eine Pause von 1 Sekunde.
+        &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Nach der Pause spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine weitere Pause von 1 Sekunde. Höre nun genau zu!
+        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine  Pause von .5 Sekunde. Höre nun genau zu!
     &lt;/div&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;5. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
@@ -706,20 +715,37 @@
 &lt;/body&gt;</t>
   </si>
   <si>
+    <t>&lt;h4&gt;Welcome to the Musical Scene Analysis (MSA) Test&lt;/h4&gt;
+    &lt;p&gt;In this test, you will be presented with a series of music excerpts. Each excerpt is structured as follows:&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Initial Music Segment (8 seconds):&lt;/strong&gt; A song will play for 8 seconds. This is the initial music segment. Please listen passively.
+    &lt;/div&gt;
+       &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Target Instrument Segment:&lt;/strong&gt; Thereafter, a single instrument (either a lead voice, bass, guitar, or piano) will play. This is the target instrument. Listen carefully!
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Pause (1 second):&lt;/strong&gt; After the target instrument segment, there will be a 0.5-second pause.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;5. Mixture Segment (2 seconds):&lt;/strong&gt; Finally, a mixture of several instruments will play for 2 seconds. This is the mixture segment. The target instrument may or may not be included in this mixture.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Your task is to determine whether the target instrument that played after the first pause is included in the final mixture segment.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Before the data collection begins, you will have the opportunity to hear some examples and do some practice trials. This will help you understand the task better and prepare you for the actual test.&lt;/p&gt;</t>
+  </si>
+  <si>
     <t>&lt;body&gt;
     &lt;h4&gt;Willkommen zum Test für Musikalische Szenenanalyse (MSA)&lt;/h4&gt;
     &lt;p&gt;In diesem Test werden Ihnen eine Reihe von Musikausschnitten präsentiert. Jeder Ausschnitt ist wie folgt strukturiert:&lt;/p&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment. Bitte hören Sie einfach passsiv zu.
     &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;2. Pause (1 Sekunde):&lt;/strong&gt; Nach dem anfänglichen Musiksegment gibt es eine Pause von 1 Sekunde.
+      &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Nach der Pause spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine weitere Pause von 1 Sekunde. Hören Sie genau zu!
+        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine Pause von .5 Sekunde. Hören Sie genau zu!
     &lt;/div&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;5. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
@@ -731,43 +757,17 @@
 &lt;/body&gt;</t>
   </si>
   <si>
-    <t>&lt;h4&gt;Welcome to the Musical Scene Analysis (MSA) Test&lt;/h4&gt;
-    &lt;p&gt;In this test, you will be presented with a series of music excerpts. Each excerpt is structured as follows:&lt;/p&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;1. Initial Music Segment (8 seconds):&lt;/strong&gt; A song will play for 8 seconds. This is the initial music segment. Please listen passively.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;2. Pause (1 second):&lt;/strong&gt; After the initial music segment, there will be a 1-second pause.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Target Instrument Segment:&lt;/strong&gt; Following the pause, a single instrument (either a lead voice, bass, guitar, or piano) will play. This is the target instrument. Listen carefully!
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 second):&lt;/strong&gt; After the target instrument segment, there will be another 1-second pause.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;5. Mixture Segment (2 seconds):&lt;/strong&gt; Finally, a mixture of several instruments will play for 2 seconds. This is the mixture segment. The target instrument may or may not be included in this mixture.
-    &lt;/div&gt;
-    &lt;div class="task"&gt;
-        &lt;strong&gt;Your task is to determine whether the target instrument that played after the first pause is included in the final mixture segment.&lt;/strong&gt;
-    &lt;/div&gt;
-    &lt;p&gt;Before the data collection begins, you will have the opportunity to hear some examples and do some practice trials. This will help you understand the task better and prepare you for the actual test.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>&lt;body&gt;
     &lt;h4&gt;Bienvenue au test d'Analyse de Scène Musicale (ASM)&lt;/h4&gt;
     &lt;p&gt;Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :&lt;/p&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;1. Segment Musical Initial (8 secondes) :&lt;/strong&gt; Une chanson jouera pendant 8 secondes. C'est le segment musical initial.
     &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;2. Pause (1 seconde) :&lt;/strong&gt; Après le segment musical initial, il y aura une pause de 1 seconde.
+      &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Segment de l'Instrument Cible :&lt;/strong&gt;  Un seul instrument jouera (soit une voix principale, une basse, une guitare, ou un piano). C'est l'instrument cible.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Segment de l'Instrument Cible :&lt;/strong&gt; Suite à la pause, un seul instrument (soit une voix principale, une basse, une guitare, ou un piano) jouera. C'est l'instrument cible.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 seconde) :&lt;/strong&gt; Après le segment de l'instrument cible, il y aura une autre pause de 1 seconde.
+        &lt;strong&gt;4. Pause (1 seconde) :&lt;/strong&gt; Après le segment de l'instrument cible, il y aura une pause de 0.5 seconde.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
         &lt;strong&gt;5. Segment de Mélange (2 secondes) :&lt;/strong&gt; Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.
@@ -777,18 +777,6 @@
     &lt;/div&gt;
        &lt;p&gt;Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.&lt;/p&gt;
 &lt;/body&gt;</t>
-  </si>
-  <si>
-    <t>de</t>
-  </si>
-  <si>
-    <t>fr</t>
-  </si>
-  <si>
-    <t>en</t>
-  </si>
-  <si>
-    <t>de_f</t>
   </si>
 </sst>
 </file>
@@ -941,7 +929,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -992,7 +980,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -1325,16 +1313,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2034,21 +2022,21 @@
         <v>173</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" ht="393.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>132</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updating MSA package number
</commit_message>
<xml_diff>
--- a/data_raw/MSA_dict.xlsx
+++ b/data_raw/MSA_dict.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Desktop\MSA test package\MSA PsychTest R package\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9739EBA-AB9E-49A9-A066-142C57589199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3089685-BBE7-4873-A320-B70B2E0C99D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="185">
   <si>
     <t>key</t>
   </si>
@@ -459,93 +459,6 @@
     <t>INSTRUCTIONS_LONG</t>
   </si>
   <si>
-    <t>Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :</t>
-  </si>
-  <si>
-    <r>
-      <t>1. Segment Musical Initial (8 secondes) :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Une chanson jouera pendant 8 secondes. C'est le segment musical initial.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2. Pause (1 seconde) :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Après le segment musical initial, il y aura une pause de 1 seconde.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>3. Segment de l'Instrument Cible :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Suite à la pause, un seul instrument (soit une voix principale, une basse, une guitare, ou un piano) jouera. C'est l'instrument cible.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>4. Pause (1 seconde) :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Après le segment de l'instrument cible, il y aura une autre pause de 1 seconde.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>5. Segment de Mélange (2 secondes) :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.</t>
-    </r>
-  </si>
-  <si>
-    <t>Votre tâche est de déterminer si l'instrument cible qui a joué après la première pause est inclus dans le segment de mélange final.</t>
-  </si>
-  <si>
-    <t>Veuillez écouter attentivement chaque segment et prendre votre décision en fonction des sons que vous entendez. Bonne chance!</t>
-  </si>
-  <si>
-    <t>Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.</t>
-  </si>
-  <si>
     <t>Des extraits musicaux vont être présentés pour ce test. Chaque extrait est en deux parties. Un extrait avec un instrument seul (voix, basse, guitare ou piano) est présenté  dans un premier temps, puis un mélange avec plusieurs instruments (Mix). \\ &lt;strong&gt; Votre tâche est de décider, si l'instrument présenté seul est aussi présent dans le mix avec plusieurs instruments. &lt;/strong&gt;\\ Le test commence et vos réponses sont enregistrées quand vous cliquez sur "suivant".</t>
   </si>
   <si>
@@ -691,6 +604,50 @@
   </si>
   <si>
     <t>de_f</t>
+  </si>
+  <si>
+    <t>&lt;body&gt;
+    &lt;h4&gt;Bienvenue au test d'Analyse de Scène Musicale (ASM)&lt;/h4&gt;
+    &lt;p&gt;Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Segment Musical Initial (8 secondes) :&lt;/strong&gt; Une chanson jouera pendant 8 secondes. C'est le segment musical initial.
+    &lt;/div&gt;
+      &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Segment de l'Instrument Cible :&lt;/strong&gt;  Un seul instrument jouera (soit une voix principale, une basse, une guitare, ou un piano). C'est l'instrument cible.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Pause (1 seconde) :&lt;/strong&gt; Après le segment de l'instrument cible, il y aura une pause de 0.5 seconde.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Segment de Mélange (2 secondes) :&lt;/strong&gt; Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Votre tâche est de déterminer si l'instrument cible qui a joué après la première pause est inclus dans le segment de mélange final.&lt;/strong&gt;
+    &lt;/div&gt;
+       &lt;p&gt;Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.&lt;/p&gt;
+&lt;/body&gt;</t>
+  </si>
+  <si>
+    <t>&lt;body&gt;
+    &lt;h4&gt;Willkommen zum Test für Musikalische Szenenanalyse (MSA)&lt;/h4&gt;
+    &lt;p&gt;In diesem Test werden Ihnen eine Reihe von Musikausschnitten präsentiert. Jeder Ausschnitt ist wie folgt strukturiert:&lt;/p&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment. Bitte hören Sie einfach passsiv zu.
+    &lt;/div&gt;
+      &lt;div class="segment"&gt;
+        &lt;strong&gt;2. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;3. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine Pause von .5 Sekunde. Hören Sie genau zu!
+    &lt;/div&gt;
+    &lt;div class="segment"&gt;
+        &lt;strong&gt;4. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
+    &lt;/div&gt;
+    &lt;div class="task"&gt;
+        &lt;strong&gt;Ihre Aufgabe besteht darin zu bestimmen, ob das Zielinstrument, das nach der ersten Pause gespielt hat, in der abschließenden Mixtur enthalten ist.&lt;/strong&gt;
+    &lt;/div&gt;
+    &lt;p&gt;Bevor die Datenerfassung beginnt, haben Sie die Möglichkeit, einige Beispiele zu hören und einige Übungsdurchläufe zu machen. Dies wird Ihnen helfen, die Aufgabe besser zu verstehen und sich auf den eigentlichen Test vorzubereiten.&lt;/p&gt;
+&lt;/body&gt;</t>
   </si>
   <si>
     <t>&lt;body&gt;
@@ -700,13 +657,13 @@
         &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment. Bitte höre einfach passiv zu.
     &lt;/div&gt;
         &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
+        &lt;strong&gt;2. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine  Pause von .5 Sekunde. Höre nun genau zu!
+        &lt;strong&gt;3. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine  Pause von .5 Sekunde. Höre nun genau zu!
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;5. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
+        &lt;strong&gt;4. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
     &lt;/div&gt;
     &lt;div class="task"&gt;
         &lt;strong&gt;Deine Aufgabe besteht darin zu bestimmen, ob das Zielinstrument, das nach der ersten Pause gespielt hat, in der abschließenden Mixtur enthalten ist.&lt;/strong&gt;
@@ -721,62 +678,18 @@
         &lt;strong&gt;1. Initial Music Segment (8 seconds):&lt;/strong&gt; A song will play for 8 seconds. This is the initial music segment. Please listen passively.
     &lt;/div&gt;
        &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Target Instrument Segment:&lt;/strong&gt; Thereafter, a single instrument (either a lead voice, bass, guitar, or piano) will play. This is the target instrument. Listen carefully!
+        &lt;strong&gt;2. Target Instrument Segment:&lt;/strong&gt; Thereafter, a single instrument (either a lead voice, bass, guitar, or piano) will play. This is the target instrument. Listen carefully!
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 second):&lt;/strong&gt; After the target instrument segment, there will be a 0.5-second pause.
+        &lt;strong&gt;3. Pause (1 second):&lt;/strong&gt; After the target instrument segment, there will be a 0.5-second pause.
     &lt;/div&gt;
     &lt;div class="segment"&gt;
-        &lt;strong&gt;5. Mixture Segment (2 seconds):&lt;/strong&gt; Finally, a mixture of several instruments will play for 2 seconds. This is the mixture segment. The target instrument may or may not be included in this mixture.
+        &lt;strong&gt;4. Mixture Segment (2 seconds):&lt;/strong&gt; Finally, a mixture of several instruments will play for 2 seconds. This is the mixture segment. The target instrument may or may not be included in this mixture.
     &lt;/div&gt;
     &lt;div class="task"&gt;
         &lt;strong&gt;Your task is to determine whether the target instrument that played after the first pause is included in the final mixture segment.&lt;/strong&gt;
     &lt;/div&gt;
     &lt;p&gt;Before the data collection begins, you will have the opportunity to hear some examples and do some practice trials. This will help you understand the task better and prepare you for the actual test.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;body&gt;
-    &lt;h4&gt;Willkommen zum Test für Musikalische Szenenanalyse (MSA)&lt;/h4&gt;
-    &lt;p&gt;In diesem Test werden Ihnen eine Reihe von Musikausschnitten präsentiert. Jeder Ausschnitt ist wie folgt strukturiert:&lt;/p&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;1. Anfängliches Musiksegment (8 Sekunden):&lt;/strong&gt; Ein Lied wird für 8 Sekunden abgespielt. Dies ist das anfängliche Musiksegment. Bitte hören Sie einfach passsiv zu.
-    &lt;/div&gt;
-      &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Zielinstrumentsegment:&lt;/strong&gt; Direkt im Anschluss spielt ein einzelnes Instrument (entweder eine Lead-Stimme, Bass, Gitarre oder Klavier). Dies ist das Zielinstrument.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 Sekunde):&lt;/strong&gt; Nach dem Zielinstrumentsegment gibt es eine Pause von .5 Sekunde. Hören Sie genau zu!
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;5. Mixtur (2 Sekunden):&lt;/strong&gt; Zuletzt spielt eine Mischung aus mehreren Instrumenten für 2 Sekunden. Dies ist die Mixtur. Das Zielinstrument kann in dieser Mixtur enthalten sein oder auch nicht.
-    &lt;/div&gt;
-    &lt;div class="task"&gt;
-        &lt;strong&gt;Ihre Aufgabe besteht darin zu bestimmen, ob das Zielinstrument, das nach der ersten Pause gespielt hat, in der abschließenden Mixtur enthalten ist.&lt;/strong&gt;
-    &lt;/div&gt;
-    &lt;p&gt;Bevor die Datenerfassung beginnt, haben Sie die Möglichkeit, einige Beispiele zu hören und einige Übungsdurchläufe zu machen. Dies wird Ihnen helfen, die Aufgabe besser zu verstehen und sich auf den eigentlichen Test vorzubereiten.&lt;/p&gt;
-&lt;/body&gt;</t>
-  </si>
-  <si>
-    <t>&lt;body&gt;
-    &lt;h4&gt;Bienvenue au test d'Analyse de Scène Musicale (ASM)&lt;/h4&gt;
-    &lt;p&gt;Dans ce test, vous serez présenté à une série d'extraits musicaux. Chaque extrait est structuré comme suit :&lt;/p&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;1. Segment Musical Initial (8 secondes) :&lt;/strong&gt; Une chanson jouera pendant 8 secondes. C'est le segment musical initial.
-    &lt;/div&gt;
-      &lt;div class="segment"&gt;
-        &lt;strong&gt;3. Segment de l'Instrument Cible :&lt;/strong&gt;  Un seul instrument jouera (soit une voix principale, une basse, une guitare, ou un piano). C'est l'instrument cible.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;4. Pause (1 seconde) :&lt;/strong&gt; Après le segment de l'instrument cible, il y aura une pause de 0.5 seconde.
-    &lt;/div&gt;
-    &lt;div class="segment"&gt;
-        &lt;strong&gt;5. Segment de Mélange (2 secondes) :&lt;/strong&gt; Finalement, un mélange de plusieurs instruments jouera pendant 2 secondes. C'est le segment de mélange. L'instrument cible peut ou ne peut pas être inclus dans ce mélange.
-    &lt;/div&gt;
-    &lt;div class="task"&gt;
-        &lt;strong&gt;Votre tâche est de déterminer si l'instrument cible qui a joué après la première pause est inclus dans le segment de mélange final.&lt;/strong&gt;
-    &lt;/div&gt;
-       &lt;p&gt;Avant que la collecte de données ne commence, vous aurez l'opportunité d'entendre quelques exemples et de faire quelques essais pratiques. Cela vous aidera à mieux comprendre la tâche et à vous préparer pour le test réel.&lt;/p&gt;
-&lt;/body&gt;</t>
   </si>
 </sst>
 </file>
@@ -929,7 +842,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -980,7 +893,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -1313,16 +1226,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="C1" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D1" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="E1" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1339,24 +1252,24 @@
         <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.25">
@@ -1373,7 +1286,7 @@
         <v>130</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1390,7 +1303,7 @@
         <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1407,7 +1320,7 @@
         <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1424,7 +1337,7 @@
         <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1441,7 +1354,7 @@
         <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1458,7 +1371,7 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1475,7 +1388,7 @@
         <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1492,7 +1405,7 @@
         <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1509,7 +1422,7 @@
         <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1526,7 +1439,7 @@
         <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1543,7 +1456,7 @@
         <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1560,7 +1473,7 @@
         <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1577,7 +1490,7 @@
         <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1594,7 +1507,7 @@
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1611,7 +1524,7 @@
         <v>34</v>
       </c>
       <c r="E18" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="75" x14ac:dyDescent="0.25">
@@ -1628,7 +1541,7 @@
         <v>95</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1684,36 +1597,36 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -1730,7 +1643,7 @@
         <v>98</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -1747,7 +1660,7 @@
         <v>97</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1764,7 +1677,7 @@
         <v>92</v>
       </c>
       <c r="E27" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1781,7 +1694,7 @@
         <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1798,7 +1711,7 @@
         <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1815,7 +1728,7 @@
         <v>101</v>
       </c>
       <c r="E30" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1832,7 +1745,7 @@
         <v>118</v>
       </c>
       <c r="E31" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1849,7 +1762,7 @@
         <v>50</v>
       </c>
       <c r="E32" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1883,7 +1796,7 @@
         <v>119</v>
       </c>
       <c r="E34" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1900,7 +1813,7 @@
         <v>56</v>
       </c>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1917,7 +1830,7 @@
         <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1951,7 +1864,7 @@
         <v>72</v>
       </c>
       <c r="E38" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1968,7 +1881,7 @@
         <v>73</v>
       </c>
       <c r="E39" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1985,7 +1898,7 @@
         <v>74</v>
       </c>
       <c r="E40" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2002,7 +1915,7 @@
         <v>88</v>
       </c>
       <c r="E41" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -2019,7 +1932,7 @@
         <v>91</v>
       </c>
       <c r="E42" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="393.75" x14ac:dyDescent="0.25">
@@ -2027,62 +1940,44 @@
         <v>132</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E45" s="3" t="s">
-        <v>133</v>
-      </c>
+      <c r="E45" s="3"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E47" s="4" t="s">
-        <v>134</v>
-      </c>
+      <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E48" s="4" t="s">
-        <v>135</v>
-      </c>
+      <c r="E48" s="4"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E49" s="4" t="s">
-        <v>136</v>
-      </c>
+      <c r="E49" s="4"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E50" s="4" t="s">
-        <v>137</v>
-      </c>
+      <c r="E50" s="4"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E51" s="4" t="s">
-        <v>138</v>
-      </c>
+      <c r="E51" s="4"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E52" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E52" s="4"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E54" s="3" t="s">
-        <v>140</v>
-      </c>
+      <c r="E54" s="3"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E56" s="3" t="s">
-        <v>141</v>
-      </c>
+      <c r="E56" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>